<commit_message>
added ability to give same user specified path to several ip addresses, as well as added ip out of range check
</commit_message>
<xml_diff>
--- a/SeppoUbuntu stationsinformation.xlsx
+++ b/SeppoUbuntu stationsinformation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2035" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2039" uniqueCount="272">
   <si>
     <t>Device</t>
   </si>
@@ -824,6 +824,12 @@
   </si>
   <si>
     <t>127.0.0.254</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>desc</t>
   </si>
 </sst>
 </file>
@@ -1155,7 +1161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K254"/>
+  <dimension ref="A1:L254"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="20.7109375" customWidth="1"/>
@@ -1166,9 +1172,10 @@
     <col min="9" max="9" width="30.7109375" customWidth="1"/>
     <col min="10" max="10" width="30.7109375" customWidth="1"/>
     <col min="11" max="11" width="30.7109375" customWidth="1"/>
+    <col min="12" max="12" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1202,8 +1209,11 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="L1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1225,8 +1235,11 @@
       <c r="H2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="L2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1248,8 +1261,11 @@
       <c r="H3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="4" spans="1:11">
+      <c r="L3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -1271,8 +1287,11 @@
       <c r="H4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="L4" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1295,7 +1314,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1318,7 +1337,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1341,7 +1360,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1364,7 +1383,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1387,7 +1406,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1410,7 +1429,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1433,7 +1452,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1456,7 +1475,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1479,7 +1498,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1502,7 +1521,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:12">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1525,7 +1544,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
         <v>31</v>
       </c>

</xml_diff>